<commit_message>
updated based on the smaller lumen diameters
</commit_message>
<xml_diff>
--- a/files/excel/channel-resistance-sv.xlsx
+++ b/files/excel/channel-resistance-sv.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,19 +491,19 @@
         <v>0.124888688130694</v>
       </c>
       <c r="E2" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F2" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>998.9948499758551</v>
+        <v>1505.724038438485</v>
       </c>
       <c r="I2" t="n">
-        <v>45.2763488395485</v>
+        <v>129.1875453530628</v>
       </c>
     </row>
     <row r="3">
@@ -522,19 +522,19 @@
         <v>0.124888688130694</v>
       </c>
       <c r="E3" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F3" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>284.379323447727</v>
+        <v>463.0473082930291</v>
       </c>
       <c r="I3" t="n">
-        <v>13.71737852440386</v>
+        <v>39.7392309478639</v>
       </c>
     </row>
     <row r="4">
@@ -553,19 +553,19 @@
         <v>0.124888688130694</v>
       </c>
       <c r="E4" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F4" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>285.5977045204621</v>
+        <v>463.618871264679</v>
       </c>
       <c r="I4" t="n">
-        <v>13.74385744411511</v>
+        <v>39.76375517481326</v>
       </c>
     </row>
     <row r="5">
@@ -584,19 +584,19 @@
         <v>0.124888688130694</v>
       </c>
       <c r="E5" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F5" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>286.4376663973558</v>
+        <v>463.9047153787925</v>
       </c>
       <c r="I5" t="n">
-        <v>13.73240747213852</v>
+        <v>39.77600723285615</v>
       </c>
     </row>
     <row r="6">
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.9</v>
+        <v>0.842</v>
       </c>
       <c r="C6" t="n">
         <v>0.049</v>
@@ -615,122 +615,114 @@
         <v>0.124888688130694</v>
       </c>
       <c r="E6" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F6" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>915.8732393831275</v>
+        <v>650.4502200046295</v>
       </c>
       <c r="I6" t="n">
-        <v>43.75523172773829</v>
+        <v>55.79483607439278</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>u_bend</t>
+          <t>arterial_seg6</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.0203</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.1595769121605731</v>
-      </c>
+        <v>1.058</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F7" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>345.0802598774359</v>
+        <v>72.5794312937964</v>
       </c>
       <c r="I7" t="n">
-        <v>27.70210019570675</v>
+        <v>20.68535044450083</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>veinous_seg1</t>
+          <t>u_bend</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.9</v>
+        <v>2.0203</v>
       </c>
       <c r="C8" t="n">
-        <v>0.096</v>
+        <v>0.08</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1748077488947327</v>
+        <v>0.1595769121605731</v>
       </c>
       <c r="E8" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F8" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>222.0057173275442</v>
+        <v>56.16172894781404</v>
       </c>
       <c r="I8" t="n">
-        <v>21.61819906859965</v>
+        <v>25.38233557668488</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>veinous_seg2</t>
+          <t>veinous_seg1</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.1748077488947327</v>
-      </c>
+        <v>0.842</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F9" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>73.88932323873441</v>
+        <v>14.74725835736848</v>
       </c>
       <c r="I9" t="n">
-        <v>6.990185777800909</v>
+        <v>8.397329627267274</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>veinous_seg3</t>
+          <t>veinous_seg2</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6</v>
+        <v>1.058</v>
       </c>
       <c r="C10" t="n">
         <v>0.096</v>
@@ -739,25 +731,25 @@
         <v>0.1748077488947327</v>
       </c>
       <c r="E10" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F10" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>69.66647911622188</v>
+        <v>156.503939743272</v>
       </c>
       <c r="I10" t="n">
-        <v>6.80609711220281</v>
+        <v>29.23627012009731</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>veinous_seg4</t>
+          <t>veinous_seg3</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -770,29 +762,29 @@
         <v>0.1748077488947327</v>
       </c>
       <c r="E11" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F11" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>70.42521024573804</v>
+        <v>109.3974729970752</v>
       </c>
       <c r="I11" t="n">
-        <v>6.841964279269075</v>
+        <v>19.31571047016119</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>veinous_seg5</t>
+          <t>veinous_seg4</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.95</v>
+        <v>0.6</v>
       </c>
       <c r="C12" t="n">
         <v>0.096</v>
@@ -801,19 +793,81 @@
         <v>0.1748077488947327</v>
       </c>
       <c r="E12" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="F12" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>237.8417174420948</v>
+        <v>109.4075417408123</v>
       </c>
       <c r="I12" t="n">
-        <v>22.60482700423628</v>
+        <v>19.31659950252111</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>veinous_seg5</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.1748077488947327</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>109.4507351579159</v>
+      </c>
+      <c r="I13" t="n">
+        <v>19.32041248619501</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>veinous_seg6</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1748077488947327</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>355.6460907263008</v>
+      </c>
+      <c r="I14" t="n">
+        <v>62.78525425134328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>